<commit_message>
package_qc: read the text of Office, PDF and JSON files
The check only scanned .html, .md and .qmd, so the stale register
spreadsheet passed CI with vendor names and "subject" in it. A new
section extracts the visible text of every published .xlsx, .docx,
.pptx, .pdf (via pdftotext) and .json file and applies the framing and
terminology checks plus a British-spelling check; em dashes are issues
in the rewritten pipeline documents and warnings elsewhere. The framing
pattern also catches the hybrid-AI and in-house program wording, the
"subject" pattern catches per-subject, subject-level, intra-/inter-subject
and subject data, and --all lists every finding.

CI installs poppler-utils for pdftotext. The two British spellings the
new check found in the UAT workbook (behaviour, labelling) are fixed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/uat_irt/UAT_IRT_RTSM_Workbook.xlsx
+++ b/uat_irt/UAT_IRT_RTSM_Workbook.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">IRT / RTSM User Acceptance Testing  —  how to run this UAT (parallel-group study)</t>
   </si>
   <si>
-    <t xml:space="preserve">UAT is your confirmation, in a TEST environment, that the vendor's randomization &amp; drug-supply build does exactly what the URS says — before a single real participant is randomized. This workbook is the tool you fill in as you go; the HTML 'UAT guide' walks the full detail with worked test scripts. As the biostatistician you OWN the confirmation that the IRT allocates per your list: right arm, right stratum, right block behaviour, concealed until dosing.</t>
+    <t xml:space="preserve">UAT is your confirmation, in a TEST environment, that the vendor's randomization &amp; drug-supply build does exactly what the URS says — before a single real participant is randomized. This workbook is the tool you fill in as you go; the HTML 'UAT guide' walks the full detail with worked test scripts. As the biostatistician you OWN the confirmation that the IRT allocates per your list: right arm, right stratum, right block behavior, concealed until dosing.</t>
   </si>
   <si>
     <t xml:space="preserve">The five sheets, in order of use</t>
@@ -486,7 +486,7 @@
     <t xml:space="preserve">URS-DSP-05</t>
   </si>
   <si>
-    <t xml:space="preserve">Blinded kit labelling</t>
+    <t xml:space="preserve">Blinded kit labeling</t>
   </si>
   <si>
     <t xml:space="preserve">Inspect kit label as a blinded role.</t>

</xml_diff>